<commit_message>
refactor(ui-pdf-theme-calc): Enhance UI components and theming
- Replaced HBox-based ribbon bar with PixelDuke's Ribbon component in PdfDocumentView.
- Integrated Material Design icons for navigation and search actions in PdfDocumentView.
- Improved search bar styling and functionality in PdfDocumentView.
- Migrated WelcomeScreen recent file row styling to CSS classes for better maintainability.
- Applied JMetro styling for a more modern look and feel, with support for dark/light themes.
- Updated XlsxImporter to parse and apply cell fill colors and text colors.
- Added icon support to signature status badges in PdfDocumentView.
</commit_message>
<xml_diff>
--- a/samples/sample_sheet.xlsx
+++ b/samples/sample_sheet.xlsx
@@ -51,8 +51,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -60,13 +62,66 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="14.0"/>
+      <b val="true"/>
+      <color rgb="FF104473"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="11.0"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="11.0"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="11.0"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="darkGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor rgb="DCEBF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="DCEBF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor rgb="F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="F0F0F0"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -81,8 +136,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true" applyNumberFormat="true">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
 </styleSheet>
 </file>
@@ -93,106 +169,106 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1" ht="18.0" customHeight="true">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="18.0" customHeight="true">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s" s="2">
         <v>1</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s" s="2">
         <v>2</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s" s="2">
         <v>3</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s" s="2">
         <v>4</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="E3" t="s" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="4" ht="18.0" customHeight="true">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s" s="3">
         <v>6</v>
       </c>
-      <c r="B4" t="n" s="0">
+      <c r="B4" t="n" s="4">
         <v>150000.0</v>
       </c>
-      <c r="C4" t="n" s="0">
+      <c r="C4" t="n" s="4">
         <v>142500.0</v>
       </c>
-      <c r="D4" s="0">
+      <c r="D4" s="4">
         <f>B4-C4</f>
       </c>
-      <c r="E4" s="0">
+      <c r="E4" s="5">
         <f>IF(B4&gt;=C4,"Under Budget","Over Budget")</f>
       </c>
     </row>
     <row r="5" ht="18.0" customHeight="true">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s" s="3">
         <v>7</v>
       </c>
-      <c r="B5" t="n" s="0">
+      <c r="B5" t="n" s="4">
         <v>80000.0</v>
       </c>
-      <c r="C5" t="n" s="0">
+      <c r="C5" t="n" s="4">
         <v>84200.0</v>
       </c>
-      <c r="D5" s="0">
+      <c r="D5" s="4">
         <f>B5-C5</f>
       </c>
-      <c r="E5" s="0">
+      <c r="E5" s="5">
         <f>IF(B5&gt;=C5,"Under Budget","Over Budget")</f>
       </c>
     </row>
     <row r="6" ht="18.0" customHeight="true">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s" s="3">
         <v>8</v>
       </c>
-      <c r="B6" t="n" s="0">
+      <c r="B6" t="n" s="4">
         <v>65000.0</v>
       </c>
-      <c r="C6" t="n" s="0">
+      <c r="C6" t="n" s="4">
         <v>61800.0</v>
       </c>
-      <c r="D6" s="0">
+      <c r="D6" s="4">
         <f>B6-C6</f>
       </c>
-      <c r="E6" s="0">
+      <c r="E6" s="5">
         <f>IF(B6&gt;=C6,"Under Budget","Over Budget")</f>
       </c>
     </row>
     <row r="7" ht="18.0" customHeight="true">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s" s="3">
         <v>9</v>
       </c>
-      <c r="B7" t="n" s="0">
+      <c r="B7" t="n" s="4">
         <v>110000.0</v>
       </c>
-      <c r="C7" t="n" s="0">
+      <c r="C7" t="n" s="4">
         <v>108900.0</v>
       </c>
-      <c r="D7" s="0">
+      <c r="D7" s="4">
         <f>B7-C7</f>
       </c>
-      <c r="E7" s="0">
+      <c r="E7" s="5">
         <f>IF(B7&gt;=C7,"Under Budget","Over Budget")</f>
       </c>
     </row>
     <row r="8" ht="18.0" customHeight="true">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s" s="6">
         <v>10</v>
       </c>
-      <c r="B8" s="0">
+      <c r="B8" s="7">
         <f>SUM(B4:B7)</f>
       </c>
-      <c r="C8" s="0">
+      <c r="C8" s="7">
         <f>SUM(C4:C7)</f>
       </c>
-      <c r="D8" s="0">
+      <c r="D8" s="7">
         <f>SUM(D4:D7)</f>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(core-ui-pdf-crypto): Enhance UI, PDF signature handling, and trust store logic
- Refactor UI button creation for better consistency and tooltip handling.
- Improve PDF signature verification to associate visual locations on pages.
- Enhance trust store manager to check issuer-principal relationships for trust anchors.
- Update error handling in MainWindow to suppress alerts for user-cancelled operations.
</commit_message>
<xml_diff>
--- a/samples/sample_sheet.xlsx
+++ b/samples/sample_sheet.xlsx
@@ -63,35 +63,35 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <sz val="14.0"/>
       <b val="true"/>
       <color rgb="FF104473"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="11.0"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="11.0"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="11.0"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="11.0"/>
       <b val="true"/>
     </font>

</xml_diff>